<commit_message>
Complete universal extraction and review workflow
</commit_message>
<xml_diff>
--- a/outputs/B_bank_errors.xlsx
+++ b/outputs/B_bank_errors.xlsx
@@ -26,8 +26,8 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Join Receipt'!$A$1:$H$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Provenance'!$A$1:$E$20</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Read me'!$A$1:$B$13</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Cell Evidence'!$A$1:$M$121</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Verification'!$A$1:$B$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Cell Evidence'!$A$1:$O$121</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Verification'!$A$1:$B$17</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Constraints'!$A$1:$H$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Repair Proposals'!$A$1:$I$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Correction History'!$A$1:$I$1</definedName>
@@ -1086,12 +1086,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D19" r:id="rId112"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId113"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F19" r:id="rId114"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A20" r:id="rId115"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B20" r:id="rId116"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId117"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D20" r:id="rId118"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId119"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F20" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D20" r:id="rId116"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1820,7 +1816,7 @@
         <v>0.98</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>0.382</v>
+        <v>0.138</v>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
@@ -2439,7 +2435,7 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>0.5649999999999999</v>
+        <v>0.303</v>
       </c>
     </row>
     <row r="4" ht="119" customHeight="1">
@@ -2574,7 +2570,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M121"/>
+  <dimension ref="A1:O121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -2590,6 +2586,8 @@
     <col width="13" customWidth="1" min="11" max="11"/>
     <col width="17" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
+    <col width="17" customWidth="1" min="14" max="14"/>
+    <col width="65" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -2658,6 +2656,16 @@
           <t>Role</t>
         </is>
       </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Location status</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Location reason</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="17" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -2703,6 +2711,16 @@
           <t>header</t>
         </is>
       </c>
+      <c r="N2" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O2" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="17" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
@@ -2748,6 +2766,16 @@
           <t>header</t>
         </is>
       </c>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O3" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="17" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
@@ -2793,6 +2821,16 @@
           <t>header</t>
         </is>
       </c>
+      <c r="N4" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O4" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="17" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
@@ -2838,6 +2876,16 @@
           <t>header</t>
         </is>
       </c>
+      <c r="N5" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O5" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="17" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
@@ -2883,6 +2931,16 @@
           <t>header</t>
         </is>
       </c>
+      <c r="N6" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O6" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="17" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
@@ -2928,6 +2986,16 @@
           <t>header</t>
         </is>
       </c>
+      <c r="N7" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O7" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="17" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
@@ -2973,6 +3041,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N8" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O8" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="17" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
@@ -3018,6 +3096,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N9" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O9" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="17" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
@@ -3063,6 +3151,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N10" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O10" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="17" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
@@ -3108,6 +3206,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N11" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O11" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="17" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
@@ -3153,6 +3261,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N12" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O12" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="17" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
@@ -3198,6 +3316,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N13" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O13" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="17" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
@@ -3243,6 +3371,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N14" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O14" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="17" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
@@ -3288,6 +3426,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N15" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O15" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="17" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
@@ -3333,6 +3481,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N16" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O16" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="17" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
@@ -3378,6 +3536,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N17" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O17" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="17" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
@@ -3423,6 +3591,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N18" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O18" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="17" customHeight="1">
       <c r="A19" s="2" t="inlineStr">
@@ -3468,6 +3646,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N19" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O19" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="17" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
@@ -3513,6 +3701,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N20" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O20" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="17" customHeight="1">
       <c r="A21" s="2" t="inlineStr">
@@ -3558,6 +3756,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N21" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O21" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="17" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
@@ -3603,6 +3811,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N22" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O22" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="17" customHeight="1">
       <c r="A23" s="2" t="inlineStr">
@@ -3648,6 +3866,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N23" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O23" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="17" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
@@ -3693,6 +3921,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N24" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O24" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="17" customHeight="1">
       <c r="A25" s="2" t="inlineStr">
@@ -3738,6 +3976,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N25" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O25" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="17" customHeight="1">
       <c r="A26" s="2" t="inlineStr">
@@ -3783,6 +4031,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N26" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O26" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="17" customHeight="1">
       <c r="A27" s="2" t="inlineStr">
@@ -3828,6 +4086,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N27" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O27" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="17" customHeight="1">
       <c r="A28" s="2" t="inlineStr">
@@ -3873,6 +4141,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N28" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O28" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="17" customHeight="1">
       <c r="A29" s="2" t="inlineStr">
@@ -3918,6 +4196,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N29" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O29" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="17" customHeight="1">
       <c r="A30" s="2" t="inlineStr">
@@ -3963,6 +4251,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N30" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O30" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="17" customHeight="1">
       <c r="A31" s="2" t="inlineStr">
@@ -4008,6 +4306,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N31" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O31" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="17" customHeight="1">
       <c r="A32" s="2" t="inlineStr">
@@ -4053,6 +4361,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N32" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O32" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="17" customHeight="1">
       <c r="A33" s="2" t="inlineStr">
@@ -4098,6 +4416,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N33" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O33" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="17" customHeight="1">
       <c r="A34" s="2" t="inlineStr">
@@ -4143,6 +4471,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N34" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O34" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="17" customHeight="1">
       <c r="A35" s="2" t="inlineStr">
@@ -4188,6 +4526,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N35" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O35" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="17" customHeight="1">
       <c r="A36" s="2" t="inlineStr">
@@ -4233,6 +4581,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N36" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O36" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="17" customHeight="1">
       <c r="A37" s="2" t="inlineStr">
@@ -4278,6 +4636,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N37" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O37" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="17" customHeight="1">
       <c r="A38" s="2" t="inlineStr">
@@ -4323,6 +4691,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N38" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O38" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="17" customHeight="1">
       <c r="A39" s="2" t="inlineStr">
@@ -4368,6 +4746,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N39" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O39" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="17" customHeight="1">
       <c r="A40" s="2" t="inlineStr">
@@ -4413,6 +4801,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N40" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O40" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="17" customHeight="1">
       <c r="A41" s="2" t="inlineStr">
@@ -4458,6 +4856,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N41" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O41" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="17" customHeight="1">
       <c r="A42" s="2" t="inlineStr">
@@ -4503,6 +4911,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N42" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O42" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="43" ht="17" customHeight="1">
       <c r="A43" s="2" t="inlineStr">
@@ -4548,6 +4966,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N43" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O43" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="44" ht="17" customHeight="1">
       <c r="A44" s="2" t="inlineStr">
@@ -4593,6 +5021,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N44" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O44" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="45" ht="17" customHeight="1">
       <c r="A45" s="2" t="inlineStr">
@@ -4638,6 +5076,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N45" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O45" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="46" ht="17" customHeight="1">
       <c r="A46" s="2" t="inlineStr">
@@ -4683,6 +5131,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N46" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O46" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="47" ht="17" customHeight="1">
       <c r="A47" s="2" t="inlineStr">
@@ -4728,6 +5186,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N47" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O47" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="48" ht="17" customHeight="1">
       <c r="A48" s="2" t="inlineStr">
@@ -4773,6 +5241,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N48" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O48" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="17" customHeight="1">
       <c r="A49" s="2" t="inlineStr">
@@ -4818,6 +5296,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N49" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O49" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="50" ht="17" customHeight="1">
       <c r="A50" s="2" t="inlineStr">
@@ -4863,6 +5351,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N50" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O50" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="51" ht="17" customHeight="1">
       <c r="A51" s="2" t="inlineStr">
@@ -4908,6 +5406,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N51" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O51" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="52" ht="17" customHeight="1">
       <c r="A52" s="2" t="inlineStr">
@@ -4953,6 +5461,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N52" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O52" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="53" ht="17" customHeight="1">
       <c r="A53" s="2" t="inlineStr">
@@ -4998,6 +5516,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N53" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O53" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="54" ht="17" customHeight="1">
       <c r="A54" s="2" t="inlineStr">
@@ -5043,6 +5571,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N54" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O54" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="55" ht="17" customHeight="1">
       <c r="A55" s="2" t="inlineStr">
@@ -5088,6 +5626,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N55" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O55" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="56" ht="17" customHeight="1">
       <c r="A56" s="2" t="inlineStr">
@@ -5133,6 +5681,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N56" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O56" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="57" ht="17" customHeight="1">
       <c r="A57" s="2" t="inlineStr">
@@ -5178,6 +5736,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N57" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O57" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="58" ht="17" customHeight="1">
       <c r="A58" s="2" t="inlineStr">
@@ -5223,6 +5791,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N58" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O58" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="59" ht="17" customHeight="1">
       <c r="A59" s="2" t="inlineStr">
@@ -5268,6 +5846,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N59" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O59" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="60" ht="17" customHeight="1">
       <c r="A60" s="2" t="inlineStr">
@@ -5313,6 +5901,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N60" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O60" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="61" ht="17" customHeight="1">
       <c r="A61" s="2" t="inlineStr">
@@ -5358,6 +5956,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N61" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O61" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="62" ht="17" customHeight="1">
       <c r="A62" s="2" t="inlineStr">
@@ -5403,6 +6011,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N62" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O62" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="63" ht="17" customHeight="1">
       <c r="A63" s="2" t="inlineStr">
@@ -5448,6 +6066,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N63" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O63" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="64" ht="17" customHeight="1">
       <c r="A64" s="2" t="inlineStr">
@@ -5493,6 +6121,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N64" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O64" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="65" ht="17" customHeight="1">
       <c r="A65" s="2" t="inlineStr">
@@ -5538,6 +6176,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N65" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O65" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="66" ht="17" customHeight="1">
       <c r="A66" s="2" t="inlineStr">
@@ -5583,6 +6231,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N66" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O66" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="67" ht="17" customHeight="1">
       <c r="A67" s="2" t="inlineStr">
@@ -5628,6 +6286,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N67" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O67" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="68" ht="17" customHeight="1">
       <c r="A68" s="2" t="inlineStr">
@@ -5673,6 +6341,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N68" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O68" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="69" ht="17" customHeight="1">
       <c r="A69" s="2" t="inlineStr">
@@ -5718,6 +6396,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N69" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O69" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="70" ht="17" customHeight="1">
       <c r="A70" s="2" t="inlineStr">
@@ -5763,6 +6451,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N70" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O70" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="71" ht="17" customHeight="1">
       <c r="A71" s="2" t="inlineStr">
@@ -5808,6 +6506,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N71" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O71" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="72" ht="17" customHeight="1">
       <c r="A72" s="2" t="inlineStr">
@@ -5853,6 +6561,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N72" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O72" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="73" ht="17" customHeight="1">
       <c r="A73" s="2" t="inlineStr">
@@ -5898,6 +6616,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N73" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O73" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="74" ht="17" customHeight="1">
       <c r="A74" s="2" t="inlineStr">
@@ -5943,6 +6671,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N74" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O74" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="75" ht="17" customHeight="1">
       <c r="A75" s="2" t="inlineStr">
@@ -5988,6 +6726,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N75" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O75" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="76" ht="17" customHeight="1">
       <c r="A76" s="2" t="inlineStr">
@@ -6033,6 +6781,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N76" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O76" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="77" ht="17" customHeight="1">
       <c r="A77" s="2" t="inlineStr">
@@ -6078,6 +6836,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N77" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O77" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="78" ht="17" customHeight="1">
       <c r="A78" s="2" t="inlineStr">
@@ -6123,6 +6891,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N78" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O78" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="79" ht="17" customHeight="1">
       <c r="A79" s="2" t="inlineStr">
@@ -6168,6 +6946,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N79" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O79" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="80" ht="17" customHeight="1">
       <c r="A80" s="2" t="inlineStr">
@@ -6213,6 +7001,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N80" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O80" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="81" ht="17" customHeight="1">
       <c r="A81" s="2" t="inlineStr">
@@ -6258,6 +7056,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N81" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O81" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="82" ht="17" customHeight="1">
       <c r="A82" s="2" t="inlineStr">
@@ -6303,6 +7111,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N82" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O82" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="83" ht="17" customHeight="1">
       <c r="A83" s="2" t="inlineStr">
@@ -6348,6 +7166,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N83" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O83" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="84" ht="17" customHeight="1">
       <c r="A84" s="2" t="inlineStr">
@@ -6393,6 +7221,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N84" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O84" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="85" ht="17" customHeight="1">
       <c r="A85" s="2" t="inlineStr">
@@ -6438,6 +7276,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N85" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O85" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="86" ht="17" customHeight="1">
       <c r="A86" s="2" t="inlineStr">
@@ -6483,6 +7331,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N86" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O86" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="87" ht="17" customHeight="1">
       <c r="A87" s="2" t="inlineStr">
@@ -6528,6 +7386,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N87" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O87" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="88" ht="17" customHeight="1">
       <c r="A88" s="2" t="inlineStr">
@@ -6573,6 +7441,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N88" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O88" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="89" ht="17" customHeight="1">
       <c r="A89" s="2" t="inlineStr">
@@ -6618,6 +7496,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N89" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O89" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="90" ht="17" customHeight="1">
       <c r="A90" s="2" t="inlineStr">
@@ -6663,6 +7551,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N90" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O90" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="91" ht="17" customHeight="1">
       <c r="A91" s="2" t="inlineStr">
@@ -6708,6 +7606,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N91" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O91" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="92" ht="17" customHeight="1">
       <c r="A92" s="2" t="inlineStr">
@@ -6753,6 +7661,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N92" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O92" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="93" ht="17" customHeight="1">
       <c r="A93" s="2" t="inlineStr">
@@ -6798,6 +7716,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N93" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O93" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="94" ht="17" customHeight="1">
       <c r="A94" s="2" t="inlineStr">
@@ -6843,6 +7771,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N94" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O94" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="95" ht="17" customHeight="1">
       <c r="A95" s="2" t="inlineStr">
@@ -6888,6 +7826,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N95" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O95" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="96" ht="17" customHeight="1">
       <c r="A96" s="2" t="inlineStr">
@@ -6933,6 +7881,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N96" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O96" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="97" ht="17" customHeight="1">
       <c r="A97" s="2" t="inlineStr">
@@ -6978,6 +7936,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N97" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O97" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="98" ht="17" customHeight="1">
       <c r="A98" s="2" t="inlineStr">
@@ -7023,6 +7991,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N98" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O98" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="99" ht="17" customHeight="1">
       <c r="A99" s="2" t="inlineStr">
@@ -7068,6 +8046,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N99" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O99" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="100" ht="17" customHeight="1">
       <c r="A100" s="2" t="inlineStr">
@@ -7113,6 +8101,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N100" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O100" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="101" ht="17" customHeight="1">
       <c r="A101" s="2" t="inlineStr">
@@ -7158,6 +8156,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N101" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O101" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="102" ht="17" customHeight="1">
       <c r="A102" s="2" t="inlineStr">
@@ -7203,6 +8211,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N102" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O102" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="103" ht="17" customHeight="1">
       <c r="A103" s="2" t="inlineStr">
@@ -7248,6 +8266,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N103" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O103" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="104" ht="17" customHeight="1">
       <c r="A104" s="2" t="inlineStr">
@@ -7293,6 +8321,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N104" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O104" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="105" ht="17" customHeight="1">
       <c r="A105" s="2" t="inlineStr">
@@ -7338,6 +8376,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N105" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O105" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="106" ht="17" customHeight="1">
       <c r="A106" s="2" t="inlineStr">
@@ -7383,6 +8431,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N106" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O106" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="107" ht="17" customHeight="1">
       <c r="A107" s="2" t="inlineStr">
@@ -7428,6 +8486,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N107" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O107" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="108" ht="17" customHeight="1">
       <c r="A108" s="2" t="inlineStr">
@@ -7473,6 +8541,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N108" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O108" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="109" ht="17" customHeight="1">
       <c r="A109" s="2" t="inlineStr">
@@ -7518,6 +8596,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N109" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O109" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="110" ht="17" customHeight="1">
       <c r="A110" s="2" t="inlineStr">
@@ -7563,6 +8651,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N110" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O110" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="111" ht="17" customHeight="1">
       <c r="A111" s="2" t="inlineStr">
@@ -7608,6 +8706,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N111" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O111" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="112" ht="17" customHeight="1">
       <c r="A112" s="2" t="inlineStr">
@@ -7653,6 +8761,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N112" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O112" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="113" ht="17" customHeight="1">
       <c r="A113" s="2" t="inlineStr">
@@ -7698,6 +8816,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N113" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O113" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="114" ht="17" customHeight="1">
       <c r="A114" s="2" t="inlineStr">
@@ -7743,6 +8871,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N114" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O114" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="115" ht="17" customHeight="1">
       <c r="A115" s="2" t="inlineStr">
@@ -7786,6 +8924,16 @@
       <c r="M115" s="2" t="inlineStr">
         <is>
           <t>extracted</t>
+        </is>
+      </c>
+      <c r="N115" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O115" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
         </is>
       </c>
     </row>
@@ -7829,6 +8977,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N116" s="2" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="O116" s="2" t="inlineStr">
+        <is>
+          <t>The extracted cell is empty; no source location is required.</t>
+        </is>
+      </c>
     </row>
     <row r="117" ht="17" customHeight="1">
       <c r="A117" s="2" t="inlineStr">
@@ -7870,6 +9028,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N117" s="2" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="O117" s="2" t="inlineStr">
+        <is>
+          <t>The extracted cell is empty; no source location is required.</t>
+        </is>
+      </c>
     </row>
     <row r="118" ht="17" customHeight="1">
       <c r="A118" s="2" t="inlineStr">
@@ -7915,6 +9083,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N118" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O118" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
+        </is>
+      </c>
     </row>
     <row r="119" ht="17" customHeight="1">
       <c r="A119" s="2" t="inlineStr">
@@ -7958,6 +9136,16 @@
       <c r="M119" s="2" t="inlineStr">
         <is>
           <t>extracted</t>
+        </is>
+      </c>
+      <c r="N119" s="2" t="inlineStr">
+        <is>
+          <t>located</t>
+        </is>
+      </c>
+      <c r="O119" s="2" t="inlineStr">
+        <is>
+          <t>At least one original reading has an exact source bounding box.</t>
         </is>
       </c>
     </row>
@@ -8001,6 +9189,16 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N120" s="2" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="O120" s="2" t="inlineStr">
+        <is>
+          <t>The extracted cell is empty; no source location is required.</t>
+        </is>
+      </c>
     </row>
     <row r="121" ht="17" customHeight="1">
       <c r="A121" s="2" t="inlineStr">
@@ -8042,9 +9240,19 @@
           <t>extracted</t>
         </is>
       </c>
+      <c r="N121" s="2" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="O121" s="2" t="inlineStr">
+        <is>
+          <t>The extracted cell is empty; no source location is required.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M121"/>
+  <autoFilter ref="A1:O121"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -8055,10 +9263,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="35" customWidth="1" min="1" max="1"/>
+    <col width="43" customWidth="1" min="1" max="1"/>
     <col width="65" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
@@ -8094,7 +9302,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>b51002132c517c47568cd3604426fbd78bd34784e544f7d2a31304f0fe1819ba</t>
+          <t>57646dd054cc1fc85cd6496f20fe76f0248b3d3435364b7553104a94069dee00</t>
         </is>
       </c>
     </row>
@@ -8133,65 +9341,117 @@
     <row r="7" ht="17" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>cells</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="n">
-        <v>114</v>
+          <t>Export type</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Draft Excel</t>
+        </is>
       </c>
     </row>
     <row r="8" ht="17" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>cells with source boxes</t>
+          <t>Non-empty exported cells</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="9" ht="17" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>equations</t>
+          <t>Cells with source boxes</t>
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>1</v>
+        <v>116</v>
       </c>
     </row>
     <row r="10" ht="17" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>equation checks</t>
+          <t>Cells requiring full-page evidence review</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>17</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11" ht="17" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>failed equation checks</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="n">
-        <v>2</v>
+          <t>Cell source-box coverage</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="12" ht="17" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
+          <t>cells</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="n">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="13" ht="17" customHeight="1">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>cells with source boxes</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="n">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="14" ht="17" customHeight="1">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>equations</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" ht="17" customHeight="1">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>equation checks</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="16" ht="17" customHeight="1">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>failed equation checks</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="17" ht="17" customHeight="1">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
           <t>proposals with multiple equations</t>
         </is>
       </c>
-      <c r="B12" s="2" t="n">
+      <c r="B17" s="2" t="n">
         <v>1</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B12"/>
+  <autoFilter ref="A1:B17"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>